<commit_message>
Add orthogonal splitting coupling paths and extend TA tail clamps
</commit_message>
<xml_diff>
--- a/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
+++ b/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc139a9c016eb4587"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R6b9e401ba69848d9"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>Splitting board V2 - KM05T</x:v>
+        <x:v>Splitting board V2 - RF-off zero-order reference</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -395,7 +395,7 @@
         <x:v>1/2 in mirror (BB05-E03 or equivalent)</x:v>
       </x:c>
       <x:c r="B13" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
@@ -427,7 +427,7 @@
         <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
       </x:c>
       <x:c r="B17" s="4" t="n">
-        <x:v>40</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
@@ -459,7 +459,7 @@
         <x:v>Newport M05 mirror mount</x:v>
       </x:c>
       <x:c r="B21" s="4" t="n">
-        <x:v>15</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
@@ -467,28 +467,28 @@
         <x:v>PBS cube 12.7 mm</x:v>
       </x:c>
       <x:c r="B22" s="4" t="n">
-        <x:v>3</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="2" t="str">
-        <x:v>PBS cube bonded to empty output RSP05 (not modelled)</x:v>
+        <x:v>RSP05 rotation mount</x:v>
       </x:c>
       <x:c r="B23" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>11</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="2" t="str">
-        <x:v>RSP05 rotation mount</x:v>
+        <x:v>S05TM09 lens adapter</x:v>
       </x:c>
       <x:c r="B24" s="4" t="n">
-        <x:v>11</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="2" t="str">
-        <x:v>S05TM09 lens adapter</x:v>
+        <x:v>SM05FCA2 fiber adapter</x:v>
       </x:c>
       <x:c r="B25" s="4" t="n">
         <x:v>5</x:v>
@@ -496,81 +496,79 @@
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2" t="str">
-        <x:v>SM05FCA2 fiber adapter</x:v>
+        <x:v>SM05L05 lens tube</x:v>
       </x:c>
       <x:c r="B26" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
-      <x:c r="A27" s="2" t="str">
-        <x:v>SM05L05 lens tube</x:v>
-      </x:c>
-      <x:c r="B27" s="4" t="n">
-        <x:v>5</x:v>
-      </x:c>
+      <x:c r="A27" s="2"/>
+      <x:c r="B27" s="4"/>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
-      <x:c r="A28" s="2"/>
-      <x:c r="B28" s="4"/>
-    </x:row>
-    <x:row r="29" ht="24" customHeight="1">
-      <x:c r="A29" s="8" t="str">
+      <x:c r="A28" s="8" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="B29" s="9"/>
+      <x:c r="B28" s="9"/>
+    </x:row>
+    <x:row r="29" ht="44" customHeight="1">
+      <x:c r="A29" s="10" t="str">
+        <x:v>1. Modelled component quantities: Splitting_Board_V2_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+      </x:c>
+      <x:c r="B29" s="4"/>
     </x:row>
     <x:row r="30" ht="44" customHeight="1">
       <x:c r="A30" s="10" t="str">
-        <x:v>1. Modelled component quantities: Splitting_Board_V2_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+        <x:v>2. Tapping classification: Splitting_Board_V2_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
       </x:c>
       <x:c r="B30" s="4"/>
     </x:row>
-    <x:row r="31" ht="44" customHeight="1">
-      <x:c r="A31" s="10" t="str">
-        <x:v>2. Tapping classification: Splitting_Board_V2_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
+    <x:row r="31" ht="24" customHeight="1">
+      <x:c r="A31" s="2" t="str">
+        <x:v>3. Plate holes: 85 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
       </x:c>
       <x:c r="B31" s="4"/>
     </x:row>
-    <x:row r="32" ht="24" customHeight="1">
-      <x:c r="A32" s="2" t="str">
-        <x:v>3. Plate holes: 77 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
+    <x:row r="32" ht="44" customHeight="1">
+      <x:c r="A32" s="10" t="str">
+        <x:v>4. AOM lower seats are integral with the baseplate. Only the upper AOM adapter is a separate part.</x:v>
       </x:c>
       <x:c r="B32" s="4"/>
     </x:row>
     <x:row r="33" ht="44" customHeight="1">
       <x:c r="A33" s="10" t="str">
-        <x:v>4. AOM lower seats are integral with the baseplate. Only the upper AOM adapter is a separate part.</x:v>
+        <x:v>5. 10 bare 8-32 taps retain the fiber tail-clamp hole pairs. They are baseplate machining; the tail clamps are not modelled parts.</x:v>
       </x:c>
       <x:c r="B33" s="4"/>
     </x:row>
     <x:row r="34" ht="44" customHeight="1">
       <x:c r="A34" s="10" t="str">
-        <x:v>5. 10 bare 8-32 taps retain the fiber tail-clamp hole pairs. They are baseplate machining; the tail clamps are not modelled parts.</x:v>
+        <x:v>6. KM05T mounts are counted once at each fiber assembly root; their mirror-mount child is not counted again. The lip adapters and optical subparts are listed separately.</x:v>
       </x:c>
       <x:c r="B34" s="4"/>
     </x:row>
-    <x:row r="35" ht="44" customHeight="1">
+    <x:row r="35" ht="62" customHeight="1">
       <x:c r="A35" s="10" t="str">
-        <x:v>6. KM05T mounts are counted once at each fiber assembly root; their mirror-mount child is not counted again. The lip adapters and optical subparts are listed separately.</x:v>
+        <x:v>7. The splitting-board optical model assumes an f ~4.5 mm fiber collimation lens in each head. C220TMD-A is the retained CAD envelope, not the specified optical prescription. Confirm the actual lens and beam size before operation.</x:v>
       </x:c>
       <x:c r="B35" s="4"/>
     </x:row>
-    <x:row r="36" ht="62" customHeight="1">
+    <x:row r="36" ht="44" customHeight="1">
       <x:c r="A36" s="10" t="str">
-        <x:v>7. The splitting-board optical model assumes an f ~4.5 mm fiber collimation lens in each head. C220TMD-A is the retained CAD envelope, not the specified optical prescription. Confirm the actual lens and beam size before operation.</x:v>
+        <x:v>8. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
       </x:c>
       <x:c r="B36" s="4"/>
     </x:row>
-    <x:row r="37" ht="44" customHeight="1">
+    <x:row r="37" ht="62" customHeight="1">
       <x:c r="A37" s="10" t="str">
-        <x:v>8. The 4 empty output RSP05 mounts each require one bonded PBS cube, listed separately because it is not modelled.</x:v>
+        <x:v>9. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
       </x:c>
       <x:c r="B37" s="4"/>
     </x:row>
     <x:row r="38" ht="44" customHeight="1">
       <x:c r="A38" s="10" t="str">
-        <x:v>9. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
       </x:c>
       <x:c r="B38" s="4"/>
     </x:row>

</xml_diff>

<commit_message>
Add dedicated entrance HWPs before all seven Splitting AOMs
</commit_message>
<xml_diff>
--- a/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
+++ b/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rc6458e65cd964b4b"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfec02abb1ded43d8"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -367,7 +367,7 @@
         <x:v>Surface_Adapter_rsp05_lip.step</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
-        <x:v>11</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -387,7 +387,7 @@
         <x:v>1/2 in half-wave (HWP) waveplate</x:v>
       </x:c>
       <x:c r="B12" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>14</x:v>
       </x:c>
     </x:row>
     <x:row r="13" ht="24" customHeight="1">
@@ -475,7 +475,7 @@
         <x:v>RSP05 rotation mount</x:v>
       </x:c>
       <x:c r="B23" s="4" t="n">
-        <x:v>11</x:v>
+        <x:v>18</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
@@ -526,7 +526,7 @@
     </x:row>
     <x:row r="31" ht="24" customHeight="1">
       <x:c r="A31" s="2" t="str">
-        <x:v>3. Plate holes: 85 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
+        <x:v>3. Plate holes: 99 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
       </x:c>
       <x:c r="B31" s="4"/>
     </x:row>
@@ -554,23 +554,29 @@
       </x:c>
       <x:c r="B35" s="4"/>
     </x:row>
-    <x:row r="36" ht="44" customHeight="1">
+    <x:row r="36" ht="62" customHeight="1">
       <x:c r="A36" s="10" t="str">
-        <x:v>8. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
+        <x:v>8. Each of the 7 AOM entrances has a dedicated HWP, RSP05 and lip adapter. The 7 downstream HWPs remain installed, giving 14 HWPs in total. The 18 RSP05 mounts include 4 bonded-PBS stages that hold cubes, not additional waveplates.</x:v>
       </x:c>
       <x:c r="B36" s="4"/>
     </x:row>
-    <x:row r="37" ht="62" customHeight="1">
+    <x:row r="37" ht="44" customHeight="1">
       <x:c r="A37" s="10" t="str">
-        <x:v>9. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+        <x:v>9. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
       </x:c>
       <x:c r="B37" s="4"/>
     </x:row>
-    <x:row r="38" ht="44" customHeight="1">
+    <x:row r="38" ht="62" customHeight="1">
       <x:c r="A38" s="10" t="str">
-        <x:v>10. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+        <x:v>10. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
       </x:c>
       <x:c r="B38" s="4"/>
+    </x:row>
+    <x:row r="39" ht="44" customHeight="1">
+      <x:c r="A39" s="10" t="str">
+        <x:v>11. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+      </x:c>
+      <x:c r="B39" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Correct TA mirror support and reserve Splitting AOM adjustment clearance
</commit_message>
<xml_diff>
--- a/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
+++ b/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rfec02abb1ded43d8"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="Rb802cdaf06af4e41"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -306,7 +306,7 @@
   <x:sheetData>
     <x:row r="1" ht="30" customHeight="1">
       <x:c r="A1" s="6" t="str">
-        <x:v>Splitting board V2 - RF-off zero-order reference</x:v>
+        <x:v>Splitting board V2</x:v>
       </x:c>
       <x:c r="B1" s="4"/>
     </x:row>
@@ -560,23 +560,29 @@
       </x:c>
       <x:c r="B36" s="4"/>
     </x:row>
-    <x:row r="37" ht="44" customHeight="1">
+    <x:row r="37" ht="98" customHeight="1">
       <x:c r="A37" s="10" t="str">
-        <x:v>9. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
+        <x:v>9. AOM upper adapters, KM100PM mounts and integral seats retain the lattice installation and depth; no deeper pockets are added. External hardware clears an ideal-pivot net rotation cone of 4 degrees with 1 mm added margin. This does not certify full combined catalogue travel: the existing adapter-to-plate clearance limits some tilt directions, as recorded in the adjustment audit.</x:v>
       </x:c>
       <x:c r="B37" s="4"/>
     </x:row>
-    <x:row r="38" ht="62" customHeight="1">
+    <x:row r="38" ht="44" customHeight="1">
       <x:c r="A38" s="10" t="str">
-        <x:v>10. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+        <x:v>10. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
       </x:c>
       <x:c r="B38" s="4"/>
     </x:row>
-    <x:row r="39" ht="44" customHeight="1">
+    <x:row r="39" ht="62" customHeight="1">
       <x:c r="A39" s="10" t="str">
-        <x:v>11. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+        <x:v>11. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
       </x:c>
       <x:c r="B39" s="4"/>
+    </x:row>
+    <x:row r="40" ht="44" customHeight="1">
+      <x:c r="A40" s="10" t="str">
+        <x:v>12. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+      </x:c>
+      <x:c r="B40" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>

<commit_message>
Add input QWP to Splitting board with verified clearance and machining
</commit_message>
<xml_diff>
--- a/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
+++ b/Production/SplittingBoardV2/Splitting_Board_V2.xlsx
@@ -2,7 +2,7 @@
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
 <x:workbook xmlns:x="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <x:sheets>
-    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R940f344b3dc64f82"/>
+    <x:sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Sheet1" sheetId="1" r:id="R696ea50e9e3b4ffe"/>
   </x:sheets>
 </x:workbook>
 </file>
@@ -367,7 +367,7 @@
         <x:v>Surface_Adapter_rsp05_lip.step</x:v>
       </x:c>
       <x:c r="B9" s="4" t="n">
-        <x:v>18</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="10" ht="24" customHeight="1">
@@ -400,95 +400,95 @@
     </x:row>
     <x:row r="14" ht="24" customHeight="1">
       <x:c r="A14" s="2" t="str">
-        <x:v>1/4-20 table bolt (baseplate fixing)</x:v>
+        <x:v>1/2 in quarter-wave (QWP) waveplate</x:v>
       </x:c>
       <x:c r="B14" s="4" t="n">
-        <x:v>4</x:v>
+        <x:v>1</x:v>
       </x:c>
     </x:row>
     <x:row r="15" ht="24" customHeight="1">
       <x:c r="A15" s="2" t="str">
-        <x:v>Fiber collimation lens, f ~4.5 mm (CAD envelope: C220TMD-A)</x:v>
+        <x:v>1/4-20 table bolt (baseplate fixing)</x:v>
       </x:c>
       <x:c r="B15" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>4</x:v>
       </x:c>
     </x:row>
     <x:row r="16" ht="24" customHeight="1">
       <x:c r="A16" s="2" t="str">
-        <x:v>G&amp;H AOMO 3100-125</x:v>
+        <x:v>Fiber collimation lens, f ~4.5 mm (CAD envelope: C220TMD-A)</x:v>
       </x:c>
       <x:c r="B16" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="17" ht="24" customHeight="1">
       <x:c r="A17" s="2" t="str">
-        <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
+        <x:v>G&amp;H AOMO 3100-125</x:v>
       </x:c>
       <x:c r="B17" s="4" t="n">
-        <x:v>56</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="18" ht="24" customHeight="1">
       <x:c r="A18" s="2" t="str">
-        <x:v>IDA12-P5 iris</x:v>
+        <x:v>HKTS-5/64 thumbscrew adjuster</x:v>
       </x:c>
       <x:c r="B18" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>56</x:v>
       </x:c>
     </x:row>
     <x:row r="19" ht="24" customHeight="1">
       <x:c r="A19" s="2" t="str">
-        <x:v>KM05T fiber port mount</x:v>
+        <x:v>IDA12-P5 iris</x:v>
       </x:c>
       <x:c r="B19" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="20" ht="24" customHeight="1">
       <x:c r="A20" s="2" t="str">
-        <x:v>KM100PM (bridged)</x:v>
+        <x:v>KM05T fiber port mount</x:v>
       </x:c>
       <x:c r="B20" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="21" ht="24" customHeight="1">
       <x:c r="A21" s="2" t="str">
-        <x:v>Newport M05 mirror mount</x:v>
+        <x:v>KM100PM (bridged)</x:v>
       </x:c>
       <x:c r="B21" s="4" t="n">
-        <x:v>23</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="22" ht="24" customHeight="1">
       <x:c r="A22" s="2" t="str">
-        <x:v>PBS cube 12.7 mm</x:v>
+        <x:v>Newport M05 mirror mount</x:v>
       </x:c>
       <x:c r="B22" s="4" t="n">
-        <x:v>7</x:v>
+        <x:v>23</x:v>
       </x:c>
     </x:row>
     <x:row r="23" ht="24" customHeight="1">
       <x:c r="A23" s="2" t="str">
-        <x:v>RSP05 rotation mount</x:v>
+        <x:v>PBS cube 12.7 mm</x:v>
       </x:c>
       <x:c r="B23" s="4" t="n">
-        <x:v>18</x:v>
+        <x:v>7</x:v>
       </x:c>
     </x:row>
     <x:row r="24" ht="24" customHeight="1">
       <x:c r="A24" s="2" t="str">
-        <x:v>S05TM09 lens adapter</x:v>
+        <x:v>RSP05 rotation mount</x:v>
       </x:c>
       <x:c r="B24" s="4" t="n">
-        <x:v>5</x:v>
+        <x:v>19</x:v>
       </x:c>
     </x:row>
     <x:row r="25" ht="24" customHeight="1">
       <x:c r="A25" s="2" t="str">
-        <x:v>SM05FCA2 fiber adapter</x:v>
+        <x:v>S05TM09 lens adapter</x:v>
       </x:c>
       <x:c r="B25" s="4" t="n">
         <x:v>5</x:v>
@@ -496,93 +496,107 @@
     </x:row>
     <x:row r="26" ht="24" customHeight="1">
       <x:c r="A26" s="2" t="str">
-        <x:v>SM05L05 lens tube</x:v>
+        <x:v>SM05FCA2 fiber adapter</x:v>
       </x:c>
       <x:c r="B26" s="4" t="n">
         <x:v>5</x:v>
       </x:c>
     </x:row>
     <x:row r="27" ht="24" customHeight="1">
-      <x:c r="A27" s="2"/>
-      <x:c r="B27" s="4"/>
+      <x:c r="A27" s="2" t="str">
+        <x:v>SM05L05 lens tube</x:v>
+      </x:c>
+      <x:c r="B27" s="4" t="n">
+        <x:v>5</x:v>
+      </x:c>
     </x:row>
     <x:row r="28" ht="24" customHeight="1">
-      <x:c r="A28" s="8" t="str">
+      <x:c r="A28" s="2"/>
+      <x:c r="B28" s="4"/>
+    </x:row>
+    <x:row r="29" ht="24" customHeight="1">
+      <x:c r="A29" s="8" t="str">
         <x:v>Notes</x:v>
       </x:c>
-      <x:c r="B28" s="9"/>
-    </x:row>
-    <x:row r="29" ht="44" customHeight="1">
-      <x:c r="A29" s="10" t="str">
-        <x:v>1. Modelled component quantities: Splitting_Board_V2_validation.json. Adapter filenames follow Production/Adapters.</x:v>
-      </x:c>
-      <x:c r="B29" s="4"/>
+      <x:c r="B29" s="9"/>
     </x:row>
     <x:row r="30" ht="44" customHeight="1">
       <x:c r="A30" s="10" t="str">
+        <x:v>1. Modelled component quantities: Splitting_Board_V2_validation.json. Adapter filenames follow Production/Adapters.</x:v>
+      </x:c>
+      <x:c r="B30" s="4"/>
+    </x:row>
+    <x:row r="31" ht="44" customHeight="1">
+      <x:c r="A31" s="10" t="str">
         <x:v>2. Tapping classification: Splitting_Board_V2_baseplate_TAP_or_NOT.pdf. Hole locations and counts come from the exported plate solid.</x:v>
       </x:c>
-      <x:c r="B30" s="4"/>
-    </x:row>
-    <x:row r="31" ht="24" customHeight="1">
-      <x:c r="A31" s="2" t="str">
-        <x:v>3. Plate holes: 99 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
-      </x:c>
       <x:c r="B31" s="4"/>
     </x:row>
-    <x:row r="32" ht="44" customHeight="1">
-      <x:c r="A32" s="10" t="str">
-        <x:v>4. AOM lower seats are integral with the baseplate. Only the upper AOM adapter is a separate part.</x:v>
+    <x:row r="32" ht="24" customHeight="1">
+      <x:c r="A32" s="2" t="str">
+        <x:v>3. Plate holes: 101 x #8-32 tapped; 4 x 1/4-20 clearance (do not tap).</x:v>
       </x:c>
       <x:c r="B32" s="4"/>
     </x:row>
     <x:row r="33" ht="44" customHeight="1">
       <x:c r="A33" s="10" t="str">
-        <x:v>5. 10 bare 8-32 taps retain the fiber tail-clamp hole pairs. They are baseplate machining; the tail clamps are not modelled parts.</x:v>
+        <x:v>4. AOM lower seats are integral with the baseplate. Only the upper AOM adapter is a separate part.</x:v>
       </x:c>
       <x:c r="B33" s="4"/>
     </x:row>
     <x:row r="34" ht="44" customHeight="1">
       <x:c r="A34" s="10" t="str">
+        <x:v>5. 10 bare 8-32 taps retain the fiber tail-clamp hole pairs. They are baseplate machining; the tail clamps are not modelled parts.</x:v>
+      </x:c>
+      <x:c r="B34" s="4"/>
+    </x:row>
+    <x:row r="35" ht="44" customHeight="1">
+      <x:c r="A35" s="10" t="str">
         <x:v>6. KM05T mounts are counted once at each fiber assembly root; their mirror-mount child is not counted again. The lip adapters and optical subparts are listed separately.</x:v>
-      </x:c>
-      <x:c r="B34" s="4"/>
-    </x:row>
-    <x:row r="35" ht="62" customHeight="1">
-      <x:c r="A35" s="10" t="str">
-        <x:v>7. The splitting-board optical model assumes an f ~4.5 mm fiber collimation lens in each head. C220TMD-A is the retained CAD envelope, not the specified optical prescription. Confirm the actual lens and beam size before operation.</x:v>
       </x:c>
       <x:c r="B35" s="4"/>
     </x:row>
     <x:row r="36" ht="62" customHeight="1">
       <x:c r="A36" s="10" t="str">
-        <x:v>8. Each of the 7 AOM entrances has a dedicated HWP, RSP05 and lip adapter. The 7 downstream HWPs remain installed, giving 14 HWPs in total. The 18 RSP05 mounts include 4 bonded-PBS stages that hold cubes, not additional waveplates.</x:v>
+        <x:v>7. The splitting-board optical model assumes an f ~4.5 mm fiber collimation lens in each head. C220TMD-A is the retained CAD envelope, not the specified optical prescription. Confirm the actual lens and beam size before operation.</x:v>
       </x:c>
       <x:c r="B36" s="4"/>
     </x:row>
-    <x:row r="37" ht="98" customHeight="1">
+    <x:row r="37" ht="62" customHeight="1">
       <x:c r="A37" s="10" t="str">
-        <x:v>9. AOM upper adapters, KM100PM mounts and integral seats retain the lattice installation and depth; no deeper pockets are added. External hardware clears an ideal-pivot net rotation cone of 4 degrees with 1 mm added margin. This does not certify full combined catalogue travel: the existing adapter-to-plate clearance limits some tilt directions, as recorded in the adjustment audit.</x:v>
+        <x:v>8. Each of the 7 AOM entrances has a dedicated HWP, RSP05 and lip adapter. The 7 downstream HWPs remain installed, giving 14 HWPs in total. The 19 RSP05 mounts include 4 bonded-PBS stages that hold cubes, not additional waveplates.</x:v>
       </x:c>
       <x:c r="B37" s="4"/>
     </x:row>
-    <x:row r="38" ht="44" customHeight="1">
+    <x:row r="38" ht="62" customHeight="1">
       <x:c r="A38" s="10" t="str">
-        <x:v>10. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
+        <x:v>9. The single input QWP has its own RSP05 and lip adapter. Input order is fiber port -&gt; steering mirror -&gt; QWP -&gt; entrance HWP -&gt; AOM; the QWP is counted separately from the fourteen HWPs.</x:v>
       </x:c>
       <x:c r="B38" s="4"/>
     </x:row>
-    <x:row r="39" ht="62" customHeight="1">
+    <x:row r="39" ht="98" customHeight="1">
       <x:c r="A39" s="10" t="str">
-        <x:v>11. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+        <x:v>10. AOM upper adapters, KM100PM mounts and integral seats retain the lattice installation and depth; no deeper pockets are added. External hardware clears an ideal-pivot net rotation cone of 4 degrees with 1 mm added margin. This does not certify full combined catalogue travel: the existing adapter-to-plate clearance limits some tilt directions, as recorded in the adjustment audit.</x:v>
       </x:c>
       <x:c r="B39" s="4"/>
     </x:row>
     <x:row r="40" ht="44" customHeight="1">
       <x:c r="A40" s="10" t="str">
-        <x:v>12. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+        <x:v>11. Optical reference: AOM RF off, straight-through zero order. RF-on first-order propagation, order rejection and fiber-coupling performance are not evaluated for this layout.</x:v>
       </x:c>
       <x:c r="B40" s="4"/>
+    </x:row>
+    <x:row r="41" ht="62" customHeight="1">
+      <x:c r="A41" s="10" t="str">
+        <x:v>12. The bonded PBS cubes are modelled and counted once above. Their modelled corner adhesive pads describe the assumed bond geometry and are not separate procurement items. Adhesive selection, bond strength and coating compatibility require assembly engineering.</x:v>
+      </x:c>
+      <x:c r="B41" s="4"/>
+    </x:row>
+    <x:row r="42" ht="44" customHeight="1">
+      <x:c r="A42" s="10" t="str">
+        <x:v>13. HKTS-5/64 adjusters are modelled separately. If supplied with the selected M05 or fiber-mount kit, do not order them twice.</x:v>
+      </x:c>
+      <x:c r="B42" s="4"/>
     </x:row>
   </x:sheetData>
   <x:pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>

</xml_diff>